<commit_message>
doc: update SQL guide and ignore build logs
</commit_message>
<xml_diff>
--- a/REGISTRO_LOGIN.xlsx
+++ b/REGISTRO_LOGIN.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\00_OFI_PRESUPUESTOS_progra\3_Entregable_web_buscador_de_metrados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9091D79-9D6E-414E-9101-97063F12C37F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E7FA539-2917-4B12-8DA5-AB0BF69576B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="97">
   <si>
     <t>AREA</t>
   </si>
@@ -341,12 +341,14 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -793,7 +795,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="33.88671875" customWidth="1"/>
@@ -1117,8 +1119,8 @@
       <c r="E14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G14" s="22" t="s">
-        <v>81</v>
+      <c r="G14" s="22">
+        <v>70761089</v>
       </c>
       <c r="H14" s="1">
         <v>1111</v>
@@ -1467,6 +1469,14 @@
         <v>93</v>
       </c>
       <c r="H29" s="1">
+        <v>1111</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="15.75" customHeight="1">
+      <c r="G30">
+        <v>46893878</v>
+      </c>
+      <c r="H30" s="1">
         <v>1111</v>
       </c>
     </row>

</xml_diff>